<commit_message>
updates to catch, minor bug fixes, creep; retros; projections
</commit_message>
<xml_diff>
--- a/assessment/data/SC11_2023assessmentInputData.xlsx
+++ b/assessment/data/SC11_2023assessmentInputData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26815"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://southpacificrfmo.sharepoint.com/sites/SPRFMOSCJackMackerelWorkingGroup/Shared Documents/Data repository/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C90E4B99-100D-43C7-9015-29E9F4E4A0DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{13840C3C-8786-40F8-81E6-DB9B74E4FE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1245" yWindow="1875" windowWidth="27870" windowHeight="15885" firstSheet="4" activeTab="4" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
+    <workbookView xWindow="4320" yWindow="375" windowWidth="20910" windowHeight="13185" activeTab="3" xr2:uid="{11C67D07-EBA6-4D97-A3E6-A5FACAECFD42}"/>
   </bookViews>
   <sheets>
     <sheet name="ageComps" sheetId="1" r:id="rId1"/>
@@ -79,7 +79,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -425,9 +425,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC02C38-8F7E-48D4-BE42-B6D35726D79C}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -447,7 +447,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2022</v>
       </c>
@@ -464,7 +464,7 @@
         <v>713428.07420515595</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2022</v>
       </c>
@@ -481,7 +481,7 @@
         <v>4976982.0308692297</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2022</v>
       </c>
@@ -498,7 +498,7 @@
         <v>236217346.08494201</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2022</v>
       </c>
@@ -515,7 +515,7 @@
         <v>28319409.913065899</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -532,7 +532,7 @@
         <v>23236195.653611101</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2022</v>
       </c>
@@ -549,7 +549,7 @@
         <v>33319993.759291999</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2022</v>
       </c>
@@ -566,7 +566,7 @@
         <v>9890154.0384073891</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2022</v>
       </c>
@@ -583,7 +583,7 @@
         <v>6222674.8769826898</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2022</v>
       </c>
@@ -600,7 +600,7 @@
         <v>4302234.0597480005</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2022</v>
       </c>
@@ -617,7 +617,7 @@
         <v>1859041.5649600199</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2022</v>
       </c>
@@ -634,7 +634,7 @@
         <v>1087831.1666944099</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2022</v>
       </c>
@@ -648,7 +648,7 @@
         <v>621513.78634288302</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -665,7 +665,7 @@
         <v>145730.41836414099</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -679,7 +679,7 @@
         <v>12951.4406524608</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2023</v>
       </c>
@@ -696,7 +696,7 @@
         <v>9054103.1556504592</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2023</v>
       </c>
@@ -713,7 +713,7 @@
         <v>17690170.1157052</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2023</v>
       </c>
@@ -730,7 +730,7 @@
         <v>7945019.1326532103</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2023</v>
       </c>
@@ -747,7 +747,7 @@
         <v>5455131.5683732498</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2023</v>
       </c>
@@ -764,7 +764,7 @@
         <v>2105603.6258868501</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2023</v>
       </c>
@@ -781,7 +781,7 @@
         <v>746163.93838185701</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2023</v>
       </c>
@@ -798,7 +798,7 @@
         <v>276903.525959372</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2023</v>
       </c>
@@ -815,7 +815,7 @@
         <v>96098.2665482952</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2023</v>
       </c>
@@ -832,7 +832,7 @@
         <v>39266.443733863402</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2023</v>
       </c>
@@ -849,7 +849,7 @@
         <v>19267.518308909199</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2023</v>
       </c>
@@ -866,7 +866,7 @@
         <v>13728.6989810415</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2023</v>
       </c>
@@ -891,9 +891,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{209B4BF9-A1A2-42A3-B429-B839E2C11906}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -913,7 +913,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2022</v>
       </c>
@@ -930,7 +930,7 @@
         <v>7.0556363525138902E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2022</v>
       </c>
@@ -947,7 +947,7 @@
         <v>0.15364775883300399</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2022</v>
       </c>
@@ -964,7 +964,7 @@
         <v>0.141202514816793</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2022</v>
       </c>
@@ -981,7 +981,7 @@
         <v>0.21780144114189101</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -998,7 +998,7 @@
         <v>0.25112074945970903</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2022</v>
       </c>
@@ -1015,7 +1015,7 @@
         <v>0.27818319716867901</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2022</v>
       </c>
@@ -1032,7 +1032,7 @@
         <v>0.54391682887692006</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2022</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>0.78487162247170295</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2022</v>
       </c>
@@ -1066,7 +1066,7 @@
         <v>0.93318641066375696</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2022</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>1.0895776874716301</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2022</v>
       </c>
@@ -1100,7 +1100,7 @@
         <v>1.2520011309435</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2022</v>
       </c>
@@ -1114,7 +1114,7 @@
         <v>1.3623050469014399</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -1131,7 +1131,7 @@
         <v>1.49030777400606</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>6.5532756773258594E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2023</v>
       </c>
@@ -1165,7 +1165,7 @@
         <v>0.20606138469661101</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2023</v>
       </c>
@@ -1182,7 +1182,7 @@
         <v>0.21712830312912301</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2023</v>
       </c>
@@ -1199,7 +1199,7 @@
         <v>0.25729518898811699</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2023</v>
       </c>
@@ -1216,7 +1216,7 @@
         <v>0.31479503362204098</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2023</v>
       </c>
@@ -1233,7 +1233,7 @@
         <v>0.40985577899551001</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2023</v>
       </c>
@@ -1250,7 +1250,7 @@
         <v>0.53053049783469997</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2023</v>
       </c>
@@ -1267,7 +1267,7 @@
         <v>0.64124228171571096</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2023</v>
       </c>
@@ -1284,7 +1284,7 @@
         <v>0.81239067953101096</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2023</v>
       </c>
@@ -1301,7 +1301,7 @@
         <v>0.98524036083265398</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2023</v>
       </c>
@@ -1318,7 +1318,7 @@
         <v>1.0746060487295199</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2023</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>1.2216415358013399</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2023</v>
       </c>
@@ -1360,9 +1360,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{045D14A7-CC75-44C0-8FF4-8DE7C82A1AA5}">
   <dimension ref="A1:F201"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1382,7 +1382,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2022</v>
       </c>
@@ -1390,7 +1390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2022</v>
       </c>
@@ -1398,7 +1398,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2022</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2022</v>
       </c>
@@ -1414,7 +1414,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -1422,7 +1422,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2022</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2022</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2022</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2022</v>
       </c>
@@ -1454,7 +1454,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2022</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2022</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2022</v>
       </c>
@@ -1478,7 +1478,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2022</v>
       </c>
@@ -1486,7 +1486,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2022</v>
       </c>
@@ -1494,7 +1494,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2022</v>
       </c>
@@ -1502,7 +1502,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2022</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2022</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2022</v>
       </c>
@@ -1526,7 +1526,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2022</v>
       </c>
@@ -1537,7 +1537,7 @@
         <v>0.84400391346799786</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2022</v>
       </c>
@@ -1548,7 +1548,7 @@
         <v>2.0814862545319999</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2022</v>
       </c>
@@ -1559,7 +1559,7 @@
         <v>1.448098801378999</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2022</v>
       </c>
@@ -1570,7 +1570,7 @@
         <v>3.4433803509629994</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2022</v>
       </c>
@@ -1581,7 +1581,7 @@
         <v>7.0573987251854895</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2022</v>
       </c>
@@ -1592,7 +1592,7 @@
         <v>67.099539412588896</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2022</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>180.1568443610085</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2022</v>
       </c>
@@ -1614,7 +1614,7 @@
         <v>530.83383787103844</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2022</v>
       </c>
@@ -1625,7 +1625,7 @@
         <v>1505.8352110159456</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2022</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>2645.3331949497906</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2022</v>
       </c>
@@ -1647,7 +1647,7 @@
         <v>4472.8204090960007</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2022</v>
       </c>
@@ -1658,7 +1658,7 @@
         <v>7031.0178238260605</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2022</v>
       </c>
@@ -1669,7 +1669,7 @@
         <v>7861.2593551683967</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2022</v>
       </c>
@@ -1680,7 +1680,7 @@
         <v>8898.3804482736996</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2022</v>
       </c>
@@ -1691,7 +1691,7 @@
         <v>10273.798294530719</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2022</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>12422.95711565368</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2022</v>
       </c>
@@ -1713,7 +1713,7 @@
         <v>14764.18103400817</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2022</v>
       </c>
@@ -1724,7 +1724,7 @@
         <v>16720.031884643759</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2022</v>
       </c>
@@ -1735,7 +1735,7 @@
         <v>15826.38400063494</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2022</v>
       </c>
@@ -1746,7 +1746,7 @@
         <v>14603.443428875671</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2022</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>13255.80864406378</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2022</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>13288.38316698497</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2022</v>
       </c>
@@ -1779,7 +1779,7 @@
         <v>14160.62337806815</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2022</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>13440.93192158907</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2022</v>
       </c>
@@ -1801,7 +1801,7 @@
         <v>12543.052278584972</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2022</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>11467.404120896632</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2022</v>
       </c>
@@ -1823,7 +1823,7 @@
         <v>9319.1220392575797</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2022</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>6509.3002217479798</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2022</v>
       </c>
@@ -1845,7 +1845,7 @@
         <v>4181.2089515872867</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2022</v>
       </c>
@@ -1856,7 +1856,7 @@
         <v>2926.7749456188481</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2022</v>
       </c>
@@ -1867,7 +1867,7 @@
         <v>1733.8936835047148</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2022</v>
       </c>
@@ -1878,7 +1878,7 @@
         <v>834.7501694498751</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2022</v>
       </c>
@@ -1889,7 +1889,7 @@
         <v>474.59459621964527</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2022</v>
       </c>
@@ -1900,7 +1900,7 @@
         <v>265.63178042539391</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2022</v>
       </c>
@@ -1911,7 +1911,7 @@
         <v>156.98012212496911</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2022</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>99.702824249864989</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2022</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>88.097877805730889</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>2022</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>58.897337264864802</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>2022</v>
       </c>
@@ -1955,7 +1955,7 @@
         <v>29.222885526327531</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>2022</v>
       </c>
@@ -1966,7 +1966,7 @@
         <v>18.81220951834149</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>2022</v>
       </c>
@@ -1977,7 +1977,7 @@
         <v>8.1371965927719891</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>2022</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>6.5671349545425146</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>2022</v>
       </c>
@@ -1999,7 +1999,7 @@
         <v>2.1407335580070002</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>2022</v>
       </c>
@@ -2010,7 +2010,7 @@
         <v>2.6844367882840001</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>2022</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>0.98722722131950702</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>2022</v>
       </c>
@@ -2029,7 +2029,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:2">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>2022</v>
       </c>
@@ -2037,7 +2037,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:2">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>2022</v>
       </c>
@@ -2045,7 +2045,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:2">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>2022</v>
       </c>
@@ -2053,7 +2053,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:2">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>2022</v>
       </c>
@@ -2061,7 +2061,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:2">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>2022</v>
       </c>
@@ -2069,7 +2069,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:2">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>2022</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:2">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>2022</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:2">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>2022</v>
       </c>
@@ -2093,7 +2093,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:2">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>2022</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:2">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>2022</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:2">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>2022</v>
       </c>
@@ -2117,7 +2117,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:2">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>2022</v>
       </c>
@@ -2125,7 +2125,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:2">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>2022</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:2">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>2022</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:2">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>2022</v>
       </c>
@@ -2149,7 +2149,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:2">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>2022</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:2">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>2022</v>
       </c>
@@ -2165,7 +2165,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:2">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>2022</v>
       </c>
@@ -2173,7 +2173,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:2">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>2022</v>
       </c>
@@ -2181,7 +2181,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:2">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>2022</v>
       </c>
@@ -2189,7 +2189,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:2">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>2022</v>
       </c>
@@ -2197,7 +2197,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:2">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>2022</v>
       </c>
@@ -2205,7 +2205,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="88" spans="1:2">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>2022</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:2">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>2022</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="1:2">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>2022</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:2">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>2022</v>
       </c>
@@ -2237,7 +2237,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:2">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>2022</v>
       </c>
@@ -2245,7 +2245,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:2">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>2022</v>
       </c>
@@ -2253,7 +2253,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:2">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>2022</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:2">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>2022</v>
       </c>
@@ -2269,7 +2269,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:2">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>2022</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="97" spans="1:2">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>2022</v>
       </c>
@@ -2285,7 +2285,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:2">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>2022</v>
       </c>
@@ -2293,7 +2293,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="99" spans="1:2">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>2022</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="100" spans="1:2">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>2022</v>
       </c>
@@ -2309,7 +2309,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="101" spans="1:2">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>2022</v>
       </c>
@@ -2317,7 +2317,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:2">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>2023</v>
       </c>
@@ -2325,7 +2325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:2">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>2023</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="104" spans="1:2">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>2023</v>
       </c>
@@ -2341,7 +2341,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="105" spans="1:2">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>2023</v>
       </c>
@@ -2349,7 +2349,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="106" spans="1:2">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>2023</v>
       </c>
@@ -2357,7 +2357,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107" spans="1:2">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>2023</v>
       </c>
@@ -2365,7 +2365,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:2">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>2023</v>
       </c>
@@ -2373,7 +2373,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="109" spans="1:2">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>2023</v>
       </c>
@@ -2381,7 +2381,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="110" spans="1:2">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>2023</v>
       </c>
@@ -2389,7 +2389,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="111" spans="1:2">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>2023</v>
       </c>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="112" spans="1:2">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>2023</v>
       </c>
@@ -2405,7 +2405,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="113" spans="1:5">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>2023</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="114" spans="1:5">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>2023</v>
       </c>
@@ -2421,7 +2421,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="115" spans="1:5">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>2023</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="116" spans="1:5">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>2023</v>
       </c>
@@ -2437,7 +2437,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="117" spans="1:5">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>2023</v>
       </c>
@@ -2445,7 +2445,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="118" spans="1:5">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>2023</v>
       </c>
@@ -2453,7 +2453,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="119" spans="1:5">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>2023</v>
       </c>
@@ -2461,7 +2461,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="120" spans="1:5">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>2023</v>
       </c>
@@ -2469,7 +2469,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="121" spans="1:5">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>2023</v>
       </c>
@@ -2477,7 +2477,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="122" spans="1:5">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>2023</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>1.0482713752079982</v>
       </c>
     </row>
-    <row r="123" spans="1:5">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>2023</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>15.834389797858391</v>
       </c>
     </row>
-    <row r="124" spans="1:5">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>2023</v>
       </c>
@@ -2510,7 +2510,7 @@
         <v>55.404069107026501</v>
       </c>
     </row>
-    <row r="125" spans="1:5">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>2023</v>
       </c>
@@ -2521,7 +2521,7 @@
         <v>103.50056487324501</v>
       </c>
     </row>
-    <row r="126" spans="1:5">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>2023</v>
       </c>
@@ -2532,7 +2532,7 @@
         <v>153.32553438855001</v>
       </c>
     </row>
-    <row r="127" spans="1:5">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>2023</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>365.07368052376501</v>
       </c>
     </row>
-    <row r="128" spans="1:5">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>2023</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>652.01312859081304</v>
       </c>
     </row>
-    <row r="129" spans="1:5">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>2023</v>
       </c>
@@ -2565,7 +2565,7 @@
         <v>1452.9502880235841</v>
       </c>
     </row>
-    <row r="130" spans="1:5">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>2023</v>
       </c>
@@ -2576,7 +2576,7 @@
         <v>3364.5062263537889</v>
       </c>
     </row>
-    <row r="131" spans="1:5">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>2023</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>6852.6998283593366</v>
       </c>
     </row>
-    <row r="132" spans="1:5">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>2023</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>11791.204807422615</v>
       </c>
     </row>
-    <row r="133" spans="1:5">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>2023</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>15841.94274695941</v>
       </c>
     </row>
-    <row r="134" spans="1:5">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>2023</v>
       </c>
@@ -2620,7 +2620,7 @@
         <v>15579.586235362796</v>
       </c>
     </row>
-    <row r="135" spans="1:5">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>2023</v>
       </c>
@@ -2631,7 +2631,7 @@
         <v>12195.146803320074</v>
       </c>
     </row>
-    <row r="136" spans="1:5">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>2023</v>
       </c>
@@ -2642,7 +2642,7 @@
         <v>10043.828170201396</v>
       </c>
     </row>
-    <row r="137" spans="1:5">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>2023</v>
       </c>
@@ -2653,7 +2653,7 @@
         <v>8482.2435561528146</v>
       </c>
     </row>
-    <row r="138" spans="1:5">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>2023</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>9048.1707114093588</v>
       </c>
     </row>
-    <row r="139" spans="1:5">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>2023</v>
       </c>
@@ -2675,7 +2675,7 @@
         <v>10478.334321673057</v>
       </c>
     </row>
-    <row r="140" spans="1:5">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>2023</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>11526.396376471999</v>
       </c>
     </row>
-    <row r="141" spans="1:5">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>2023</v>
       </c>
@@ -2697,7 +2697,7 @@
         <v>12553.893553981026</v>
       </c>
     </row>
-    <row r="142" spans="1:5">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>2023</v>
       </c>
@@ -2708,7 +2708,7 @@
         <v>12059.017086579848</v>
       </c>
     </row>
-    <row r="143" spans="1:5">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>2023</v>
       </c>
@@ -2719,7 +2719,7 @@
         <v>10563.476988400071</v>
       </c>
     </row>
-    <row r="144" spans="1:5">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>2023</v>
       </c>
@@ -2730,7 +2730,7 @@
         <v>9367.6126820652498</v>
       </c>
     </row>
-    <row r="145" spans="1:5">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>2023</v>
       </c>
@@ -2741,7 +2741,7 @@
         <v>7940.2236225991546</v>
       </c>
     </row>
-    <row r="146" spans="1:5">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>2023</v>
       </c>
@@ -2752,7 +2752,7 @@
         <v>6833.66843858021</v>
       </c>
     </row>
-    <row r="147" spans="1:5">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>2023</v>
       </c>
@@ -2763,7 +2763,7 @@
         <v>6126.3496024437463</v>
       </c>
     </row>
-    <row r="148" spans="1:5">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>2023</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>4805.1197599560237</v>
       </c>
     </row>
-    <row r="149" spans="1:5">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>2023</v>
       </c>
@@ -2785,7 +2785,7 @@
         <v>3532.8842942541623</v>
       </c>
     </row>
-    <row r="150" spans="1:5">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>2023</v>
       </c>
@@ -2796,7 +2796,7 @@
         <v>2244.1986933776889</v>
       </c>
     </row>
-    <row r="151" spans="1:5">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>2023</v>
       </c>
@@ -2807,7 +2807,7 @@
         <v>1368.0406216002079</v>
       </c>
     </row>
-    <row r="152" spans="1:5">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>2023</v>
       </c>
@@ -2818,7 +2818,7 @@
         <v>768.86001062078594</v>
       </c>
     </row>
-    <row r="153" spans="1:5">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>2023</v>
       </c>
@@ -2829,7 +2829,7 @@
         <v>442.781987263627</v>
       </c>
     </row>
-    <row r="154" spans="1:5">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>2023</v>
       </c>
@@ -2840,7 +2840,7 @@
         <v>162.5021226419461</v>
       </c>
     </row>
-    <row r="155" spans="1:5">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>2023</v>
       </c>
@@ -2851,7 +2851,7 @@
         <v>98.272196893723404</v>
       </c>
     </row>
-    <row r="156" spans="1:5">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>2023</v>
       </c>
@@ -2862,7 +2862,7 @@
         <v>30.611548196208499</v>
       </c>
     </row>
-    <row r="157" spans="1:5">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>2023</v>
       </c>
@@ -2873,7 +2873,7 @@
         <v>8.5747904587909698</v>
       </c>
     </row>
-    <row r="158" spans="1:5">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>2023</v>
       </c>
@@ -2884,7 +2884,7 @@
         <v>5.1372235356665099</v>
       </c>
     </row>
-    <row r="159" spans="1:5">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>2023</v>
       </c>
@@ -2895,7 +2895,7 @@
         <v>1.8702607624405001</v>
       </c>
     </row>
-    <row r="160" spans="1:5">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>2023</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="161" spans="1:2">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>2023</v>
       </c>
@@ -2911,7 +2911,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="162" spans="1:2">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>2023</v>
       </c>
@@ -2919,7 +2919,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="163" spans="1:2">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>2023</v>
       </c>
@@ -2927,7 +2927,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="164" spans="1:2">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>2023</v>
       </c>
@@ -2935,7 +2935,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="165" spans="1:2">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>2023</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="166" spans="1:2">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>2023</v>
       </c>
@@ -2951,7 +2951,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="167" spans="1:2">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>2023</v>
       </c>
@@ -2959,7 +2959,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="168" spans="1:2">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>2023</v>
       </c>
@@ -2967,7 +2967,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="169" spans="1:2">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>2023</v>
       </c>
@@ -2975,7 +2975,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="170" spans="1:2">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>2023</v>
       </c>
@@ -2983,7 +2983,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="171" spans="1:2">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>2023</v>
       </c>
@@ -2991,7 +2991,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="172" spans="1:2">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>2023</v>
       </c>
@@ -2999,7 +2999,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="173" spans="1:2">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>2023</v>
       </c>
@@ -3007,7 +3007,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="174" spans="1:2">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>2023</v>
       </c>
@@ -3015,7 +3015,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="175" spans="1:2">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>2023</v>
       </c>
@@ -3023,7 +3023,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="176" spans="1:2">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>2023</v>
       </c>
@@ -3031,7 +3031,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="177" spans="1:2">
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>2023</v>
       </c>
@@ -3039,7 +3039,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="178" spans="1:2">
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>2023</v>
       </c>
@@ -3047,7 +3047,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="179" spans="1:2">
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>2023</v>
       </c>
@@ -3055,7 +3055,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="180" spans="1:2">
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>2023</v>
       </c>
@@ -3063,7 +3063,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="181" spans="1:2">
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>2023</v>
       </c>
@@ -3071,7 +3071,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="182" spans="1:2">
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>2023</v>
       </c>
@@ -3079,7 +3079,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="183" spans="1:2">
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>2023</v>
       </c>
@@ -3087,7 +3087,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="184" spans="1:2">
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>2023</v>
       </c>
@@ -3095,7 +3095,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="185" spans="1:2">
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>2023</v>
       </c>
@@ -3103,7 +3103,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="186" spans="1:2">
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>2023</v>
       </c>
@@ -3111,7 +3111,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="187" spans="1:2">
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>2023</v>
       </c>
@@ -3119,7 +3119,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="188" spans="1:2">
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>2023</v>
       </c>
@@ -3127,7 +3127,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="189" spans="1:2">
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>2023</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="190" spans="1:2">
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>2023</v>
       </c>
@@ -3143,7 +3143,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="191" spans="1:2">
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>2023</v>
       </c>
@@ -3151,7 +3151,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="192" spans="1:2">
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>2023</v>
       </c>
@@ -3159,7 +3159,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="193" spans="1:2">
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>2023</v>
       </c>
@@ -3167,7 +3167,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="194" spans="1:2">
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>2023</v>
       </c>
@@ -3175,7 +3175,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="195" spans="1:2">
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>2023</v>
       </c>
@@ -3183,7 +3183,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="196" spans="1:2">
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>2023</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="197" spans="1:2">
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>2023</v>
       </c>
@@ -3199,7 +3199,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="198" spans="1:2">
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>2023</v>
       </c>
@@ -3207,7 +3207,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="199" spans="1:2">
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>2023</v>
       </c>
@@ -3215,7 +3215,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="200" spans="1:2">
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>2023</v>
       </c>
@@ -3223,7 +3223,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="201" spans="1:2">
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>2023</v>
       </c>
@@ -3239,9 +3239,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7886E624-8038-4FB5-9240-586936FC87C7}">
   <dimension ref="A1:E55"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3258,72 +3258,72 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1970</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1971</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1972</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1973</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1974</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1975</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1976</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1977</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1978</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1979</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1980</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1981</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1982</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1983</v>
       </c>
@@ -3331,435 +3331,435 @@
         <v>0.832510731465533</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1984</v>
       </c>
       <c r="C16">
-        <v>0.77328348460413576</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
+        <v>0.76555064975809439</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>1985</v>
       </c>
       <c r="C17">
-        <v>0.68308603600066609</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
+        <v>0.66949262388425279</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>1986</v>
       </c>
       <c r="C18">
-        <v>0.58072905434996736</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
+        <v>0.5634808207067189</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1987</v>
       </c>
       <c r="C19">
-        <v>0.68933883136044727</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3">
+        <v>0.6621761309429085</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1988</v>
       </c>
       <c r="C20">
-        <v>0.61152501978970331</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
+        <v>0.5815542090849084</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1989</v>
       </c>
       <c r="C21">
-        <v>0.60145810362458518</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
+        <v>0.5662608652589165</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1990</v>
       </c>
       <c r="C22">
-        <v>0.52041964151318509</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
+        <v>0.48506511422461784</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1991</v>
       </c>
       <c r="C23">
-        <v>0.57972996353576056</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
+        <v>0.53494274805351461</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1992</v>
       </c>
       <c r="C24">
-        <v>0.53629921595146257</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
+        <v>0.48991858358361473</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1993</v>
       </c>
       <c r="C25">
-        <v>0.48552436619217271</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
+        <v>0.43909953376421168</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1994</v>
       </c>
       <c r="C26">
-        <v>0.5270907404155396</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
+        <v>0.47192450335958341</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1995</v>
       </c>
       <c r="C27">
-        <v>0.4755982930292772</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
+        <v>0.42156313195516587</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1996</v>
       </c>
       <c r="C28">
-        <v>0.47437137829655601</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
+        <v>0.41627085716422413</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1997</v>
       </c>
       <c r="C29">
-        <v>0.39289590267625318</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
+        <v>0.34132667030408287</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>1998</v>
       </c>
       <c r="C30">
-        <v>0.33704868717487563</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
+        <v>0.28988153932562982</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>1999</v>
       </c>
       <c r="C31">
-        <v>0.34702987823037729</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
+        <v>0.29548128662136308</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2000</v>
       </c>
       <c r="C32">
-        <v>0.33903998155477127</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
+        <v>0.2857914447366065</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2001</v>
       </c>
       <c r="C33">
-        <v>0.40785942799973102</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
+        <v>0.34036430540293661</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2002</v>
       </c>
       <c r="C34">
-        <v>0.35682001613922443</v>
+        <v>0.29479350169073476</v>
       </c>
       <c r="D34">
         <v>4.0695343769888597</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2003</v>
       </c>
       <c r="C35">
-        <v>0.317826066567508</v>
+        <v>0.25995214479480405</v>
       </c>
       <c r="D35">
-        <v>4.8817552316689898</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5">
+        <v>4.8329376793523</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2004</v>
       </c>
       <c r="C36">
-        <v>0.34671410484437842</v>
+        <v>0.2807440729978804</v>
       </c>
       <c r="D36">
-        <v>5.2933128244855796</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5">
+        <v>5.1879758992783165</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2005</v>
       </c>
       <c r="C37">
-        <v>0.31860118102728968</v>
+        <v>0.25540045257474242</v>
       </c>
       <c r="D37">
-        <v>4.2283950393612999</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5">
+        <v>4.1028074782972297</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2006</v>
       </c>
       <c r="C38">
-        <v>0.34900360739524477</v>
+        <v>0.27697424787202868</v>
       </c>
       <c r="D38">
-        <v>5.6456570958232701</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5">
+        <v>5.423195680076021</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2007</v>
       </c>
       <c r="C39">
-        <v>0.26399849962513289</v>
+        <v>0.20741785036136962</v>
       </c>
       <c r="D39">
-        <v>7.8585266207506104</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5">
+        <v>7.4733806232081008</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2008</v>
       </c>
       <c r="C40">
-        <v>0.17522631479957529</v>
+        <v>0.13629477037990842</v>
       </c>
       <c r="D40">
-        <v>4.0277767369508801</v>
+        <v>3.7920718440583863</v>
       </c>
       <c r="E40">
         <v>1680</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2009</v>
       </c>
       <c r="C41">
-        <v>0.14673263254725449</v>
+        <v>0.11299045795895972</v>
       </c>
       <c r="D41">
-        <v>1.4388040986274899</v>
+        <v>1.3410594427572344</v>
       </c>
       <c r="E41">
         <v>1185</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2010</v>
       </c>
       <c r="C42">
-        <v>0.1140641584846718</v>
+        <v>8.6955980188922893E-2</v>
       </c>
       <c r="D42">
-        <v>2.7032650048358202</v>
+        <v>2.4944234408449186</v>
       </c>
       <c r="E42">
         <v>824</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2011</v>
       </c>
       <c r="C43">
-        <v>6.3785181075663097E-2</v>
+        <v>4.8139906395579073E-2</v>
       </c>
       <c r="D43">
-        <v>6.9787049248789996</v>
+        <v>6.3751673139759912</v>
       </c>
       <c r="E43">
         <v>732</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2012</v>
       </c>
       <c r="C44">
-        <v>0.19629275324406201</v>
+        <v>0.14666446754348098</v>
       </c>
       <c r="D44">
-        <v>6.1461806421941603</v>
+        <v>5.5584956025665004</v>
       </c>
       <c r="E44">
         <v>618</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2013</v>
       </c>
       <c r="C45">
-        <v>0.17381307121944861</v>
+        <v>0.12856959368078985</v>
       </c>
       <c r="D45">
-        <v>2.7347098473804801</v>
+        <v>2.4484903406577594</v>
       </c>
       <c r="E45">
         <v>719</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2014</v>
       </c>
       <c r="C46">
-        <v>0.13889312738008519</v>
+        <v>0.10171190520227381</v>
       </c>
       <c r="D46">
-        <v>3.7120314520745299</v>
+        <v>3.2902885224533187</v>
       </c>
       <c r="E46">
         <v>760</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2015</v>
       </c>
       <c r="C47">
-        <v>0.11526353732357961</v>
+        <v>8.3563798012539298E-2</v>
       </c>
       <c r="D47">
-        <v>3.0164000257817598</v>
+        <v>2.6469544363981226</v>
       </c>
       <c r="E47">
         <v>1035</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2016</v>
       </c>
       <c r="C48">
-        <v>0.20910165002501141</v>
+        <v>0.15007863863962947</v>
       </c>
       <c r="D48">
-        <v>2.6155741965886699</v>
+        <v>2.2722691312729908</v>
       </c>
       <c r="E48">
         <v>743</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2017</v>
       </c>
       <c r="C49">
-        <v>0.25112097001249772</v>
+        <v>0.17843481567812872</v>
       </c>
       <c r="D49">
-        <v>3.3680201361499398</v>
+        <v>2.8966938566958449</v>
       </c>
       <c r="E49">
         <v>916</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2018</v>
       </c>
       <c r="C50">
-        <v>0.16377114939393159</v>
+        <v>0.11520443754859125</v>
       </c>
       <c r="D50">
-        <v>9.6985171133726595</v>
+        <v>8.2578777642777901</v>
       </c>
       <c r="E50">
         <v>807</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2019</v>
       </c>
       <c r="C51">
-        <v>0.28263162867951269</v>
+        <v>0.19682840205129151</v>
       </c>
       <c r="D51">
-        <v>16.318611520401401</v>
+        <v>13.755662506598892</v>
       </c>
       <c r="E51">
         <v>975</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2020</v>
       </c>
       <c r="C52">
-        <v>0.37255472704360459</v>
+        <v>0.25685751599641693</v>
       </c>
       <c r="D52">
-        <v>17.906153200649602</v>
+        <v>14.942931260575619</v>
       </c>
       <c r="E52">
         <v>1373</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2021</v>
       </c>
       <c r="C53">
-        <v>0.39673838877881168</v>
+        <v>0.2707956102779952</v>
       </c>
       <c r="D53">
-        <v>21.862445492912801</v>
+        <v>18.062066506560289</v>
       </c>
       <c r="E53">
         <v>1714</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2022</v>
       </c>
       <c r="C54">
-        <v>0.40878897324379532</v>
+        <v>0.27623058415635926</v>
       </c>
       <c r="D54">
-        <v>27.720055428230001</v>
+        <v>22.672425645329092</v>
       </c>
       <c r="E54">
         <v>3032</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2023</v>
       </c>
       <c r="C55">
-        <v>0.41850988778127762</v>
+        <v>0.27997129560784073</v>
       </c>
       <c r="D55">
-        <v>23.621095271521401</v>
+        <v>19.126659119260268</v>
       </c>
     </row>
   </sheetData>
@@ -3770,9 +3770,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E42CCE45-3DDC-4861-A006-F4C4C7145E6D}">
   <dimension ref="A1:G27"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3795,7 +3795,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2023</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2023</v>
       </c>
@@ -3820,7 +3820,7 @@
         <v>314185.36619066278</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2023</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>13464</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2023</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>41163</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2023</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>24149</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2023</v>
       </c>
@@ -3888,7 +3888,7 @@
         <v>70593</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2023</v>
       </c>
@@ -3905,7 +3905,7 @@
         <v>100661</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2023</v>
       </c>
@@ -3922,7 +3922,7 @@
         <v>141210</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2023</v>
       </c>
@@ -3939,7 +3939,7 @@
         <v>145699</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2023</v>
       </c>
@@ -3956,7 +3956,7 @@
         <v>79393</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2023</v>
       </c>
@@ -3970,7 +3970,7 @@
         <v>85635</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2023</v>
       </c>
@@ -3984,7 +3984,7 @@
         <v>9359</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2023</v>
       </c>
@@ -3998,7 +3998,7 @@
         <v>30581</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2023</v>
       </c>
@@ -4009,7 +4009,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2023</v>
       </c>
@@ -4023,7 +4023,7 @@
         <v>0.15893320018150198</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2023</v>
       </c>
@@ -4040,7 +4040,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2023</v>
       </c>
@@ -4057,7 +4057,7 @@
         <v>0.24399999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2023</v>
       </c>
@@ -4074,7 +4074,7 @@
         <v>0.29099999999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2023</v>
       </c>
@@ -4091,7 +4091,7 @@
         <v>0.82099999999999995</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2023</v>
       </c>
@@ -4108,7 +4108,7 @@
         <v>0.98299999999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2023</v>
       </c>
@@ -4125,7 +4125,7 @@
         <v>1.169</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2023</v>
       </c>
@@ -4142,7 +4142,7 @@
         <v>1.319</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2023</v>
       </c>
@@ -4159,7 +4159,7 @@
         <v>1.431</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2023</v>
       </c>
@@ -4173,7 +4173,7 @@
         <v>1.4870000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2023</v>
       </c>
@@ -4187,7 +4187,7 @@
         <v>1.3859999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2023</v>
       </c>
@@ -4407,13 +4407,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{228CE105-4287-40ED-B72B-E33A77B67D61}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{314ABCD6-81B4-41F5-9CBB-C1381E9CDE39}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{314ABCD6-81B4-41F5-9CBB-C1381E9CDE39}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f419981a-ca0a-4e56-9512-575f16b7ea2d"/>
+    <ds:schemaRef ds:uri="5ce05999-5605-4258-98fc-62ff4522b5fb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2AFB9C7-A01A-423B-A442-B6889BA2E519}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="99586898-a167-430f-9bd8-1309c133fb37"/>
+    <ds:schemaRef ds:uri="106056fc-f9c8-4d4e-b594-b9dbfe683f46"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>